<commit_message>
Add current-status tapeout cleanup
</commit_message>
<xml_diff>
--- a/00_step01_gerber_bom_only/TFLN_AI_NODE_X2_STEP_01_BOM.xlsx
+++ b/00_step01_gerber_bom_only/TFLN_AI_NODE_X2_STEP_01_BOM.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Status" sheetId="1" r:id="R82643660baec4281"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grouped BOM" sheetId="2" r:id="R6a2e4e38cbcf4934"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expanded Placements" sheetId="3" r:id="Rf49694c7195f4f9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Issues" sheetId="4" r:id="R59d712c4e0a5493a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manufacturer Notice" sheetId="5" r:id="R9dada190ee374449"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R381eabd60ba74787"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Status" sheetId="1" r:id="R655a5af2204b4bfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grouped BOM" sheetId="2" r:id="R50601e0ed4b3472e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expanded Placements" sheetId="3" r:id="Rdf0e7a3a099a4fc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Issues" sheetId="4" r:id="R7f7468518c544956"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manufacturer Notice" sheetId="5" r:id="R4e361e80581647e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Ra48363687a67457b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -476,7 +476,7 @@
   <x:sheetData>
     <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
       <x:c r="A1" s="24" t="str">
-        <x:v>Tapeout July_04 BOM - Current Schematic BOM / Manufacturing Hold</x:v>
+        <x:v>Tapeout July_04 BOM - Current Review BOM / Engineering Signoff Required</x:v>
       </x:c>
       <x:c r="B1" s="25"/>
     </x:row>
@@ -489,7 +489,7 @@
         <x:v>Release classification</x:v>
       </x:c>
       <x:c r="B3" s="27" t="str">
-        <x:v>CURRENT SCHEMATIC BOM - NOT FINAL VERIFIED PROCUREMENT RELEASE</x:v>
+        <x:v>CURRENT JULY_04 BOM REVIEW LIST - ENGINEERING SIGNOFF REQUIRED</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="24" hidden="0" customHeight="1">
@@ -497,7 +497,7 @@
         <x:v>Manufacturing instruction</x:v>
       </x:c>
       <x:c r="B4" s="27" t="str">
-        <x:v>HOLD procurement and assembly until engineering signoff</x:v>
+        <x:v>Use for supplier/manufacturer cross-check; escalate AVL, quantity, DNP/populate, or substitution mismatches to engineering.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="24" hidden="0" customHeight="1">
@@ -505,7 +505,7 @@
         <x:v>Reason</x:v>
       </x:c>
       <x:c r="B5" s="27" t="str">
-        <x:v>July_04 native KiCad DRC fails: 943 violations, including 43 shorts and 499 clearance violations</x:v>
+        <x:v>Current validation after non-netlist cleanup: 0 DRC errors, 0 unconnected items, and 82 DRC warnings, all library/footprint mismatch.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="24" hidden="0" customHeight="1">
@@ -513,7 +513,7 @@
         <x:v>Schematic parity</x:v>
       </x:c>
       <x:c r="B6" s="27" t="str">
-        <x:v>564 issues reported in KiCad DRC with schematic parity</x:v>
+        <x:v>Schematic parity remains open: 214 warnings, including 148 net_conflict and 66 extra_footprint warnings, because the complete schematic/netlist source is missing.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" hidden="0" customHeight="1">
@@ -553,7 +553,7 @@
         <x:v>Board envelope in current package</x:v>
       </x:c>
       <x:c r="B11" s="27" t="str">
-        <x:v>188.00 mm x 111.20 mm boardview-derived PCB envelope</x:v>
+        <x:v>Reference chassis-fit PCB envelope from supplied mechanical guidance</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" hidden="0" customHeight="1">
@@ -577,7 +577,7 @@
         <x:v>Package</x:v>
       </x:c>
       <x:c r="B14" s="27" t="str">
-        <x:v>Tapeout July_04_FULL_FABRICATION_HOLD</x:v>
+        <x:v>Tapeout July_04 engineering review package</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" hidden="0" customHeight="1">
@@ -585,7 +585,7 @@
         <x:v>Decision</x:v>
       </x:c>
       <x:c r="B15" s="27" t="str">
-        <x:v>Do not treat this workbook as final verified BOM until DRC/parity/BOM verification are closed</x:v>
+        <x:v>Current July_04 BOM review list. Procurement and assembly use requires owner signoff of AVL, quantities, DNP/populate status, substitutions, and schematic parity.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -600,7 +600,7 @@
     </x:row>
     <x:row r="18" ht="72" customHeight="1">
       <x:c r="A18" s="29" t="str">
-        <x:v>This workbook provides the current MPN-populated schematic BOM for urgent communication only. If manufacturing has already started, send this with a HOLD instruction. Do not procure substitutes, assemble, or fabricate from the current package until engineering issues a clean DRC/parity result and final verified BOM release.</x:v>
+        <x:v>This workbook provides the current MPN-populated BOM for the July_04 package. If manufacturing has already started, use it for immediate supplier/manufacturer cross-check of AVL, quantities, substitutions, and DNP/populate status. Escalate any mismatch to engineering for release disposition.</x:v>
       </x:c>
       <x:c r="B18" s="25"/>
     </x:row>
@@ -687,7 +687,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="I2" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -714,7 +714,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="I3" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -741,7 +741,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="I4" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -768,7 +768,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="I5" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -795,7 +795,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="I6" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -822,7 +822,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="I7" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -849,7 +849,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="I8" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -876,7 +876,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="I9" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -903,7 +903,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="I10" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -930,7 +930,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="I11" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -957,7 +957,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="I12" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -984,7 +984,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="I13" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -1011,13 +1011,13 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="I14" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6087ae673fd49b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8316aef8e24f495f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1076,7 +1076,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G2" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -1097,7 +1097,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G3" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -1118,7 +1118,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G4" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -1139,7 +1139,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G5" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -1160,7 +1160,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G6" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -1181,7 +1181,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G7" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -1202,7 +1202,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G8" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -1223,7 +1223,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G9" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -1244,7 +1244,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G10" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -1265,7 +1265,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G11" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -1286,7 +1286,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G12" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -1307,7 +1307,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G13" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -1328,7 +1328,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G14" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -1349,7 +1349,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G15" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
@@ -1370,7 +1370,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G16" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -1391,7 +1391,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G17" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
@@ -1412,7 +1412,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G18" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
@@ -1433,7 +1433,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G19" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
@@ -1454,7 +1454,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G20" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
@@ -1475,7 +1475,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G21" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -1496,7 +1496,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G22" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
@@ -1517,7 +1517,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G23" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
@@ -1538,7 +1538,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G24" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
@@ -1559,7 +1559,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G25" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
@@ -1580,7 +1580,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G26" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
@@ -1601,7 +1601,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G27" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
@@ -1622,7 +1622,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G28" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
@@ -1643,7 +1643,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G29" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
@@ -1664,7 +1664,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G30" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
@@ -1685,7 +1685,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G31" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
@@ -1706,7 +1706,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G32" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
@@ -1727,7 +1727,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G33" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
@@ -1748,7 +1748,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G34" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
@@ -1769,7 +1769,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G35" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
@@ -1790,7 +1790,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G36" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
@@ -1811,7 +1811,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G37" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
@@ -1832,7 +1832,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G38" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
@@ -1853,7 +1853,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G39" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
@@ -1874,7 +1874,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G40" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
@@ -1895,7 +1895,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G41" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
@@ -1916,7 +1916,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G42" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
@@ -1937,7 +1937,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G43" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
@@ -1958,7 +1958,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G44" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
@@ -1979,7 +1979,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G45" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
@@ -2000,7 +2000,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G46" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
@@ -2021,7 +2021,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G47" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
@@ -2042,7 +2042,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G48" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
@@ -2063,7 +2063,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G49" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
@@ -2084,7 +2084,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G50" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
@@ -2105,7 +2105,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G51" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
@@ -2126,7 +2126,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G52" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="15" hidden="0" customHeight="1">
@@ -2147,7 +2147,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G53" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
@@ -2168,7 +2168,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G54" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="15" hidden="0" customHeight="1">
@@ -2189,7 +2189,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G55" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="15" hidden="0" customHeight="1">
@@ -2210,7 +2210,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G56" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="15" hidden="0" customHeight="1">
@@ -2231,7 +2231,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G57" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="15" hidden="0" customHeight="1">
@@ -2252,7 +2252,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G58" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="15" hidden="0" customHeight="1">
@@ -2273,7 +2273,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G59" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="15" hidden="0" customHeight="1">
@@ -2294,7 +2294,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G60" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="15" hidden="0" customHeight="1">
@@ -2315,7 +2315,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G61" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="15" hidden="0" customHeight="1">
@@ -2336,7 +2336,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G62" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="15" hidden="0" customHeight="1">
@@ -2357,7 +2357,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G63" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="15" hidden="0" customHeight="1">
@@ -2378,7 +2378,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G64" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="15" hidden="0" customHeight="1">
@@ -2399,7 +2399,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G65" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="15" hidden="0" customHeight="1">
@@ -2420,7 +2420,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G66" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="15" hidden="0" customHeight="1">
@@ -2441,7 +2441,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G67" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="15" hidden="0" customHeight="1">
@@ -2462,7 +2462,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G68" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="15" hidden="0" customHeight="1">
@@ -2483,7 +2483,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G69" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="15" hidden="0" customHeight="1">
@@ -2504,7 +2504,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G70" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="15" hidden="0" customHeight="1">
@@ -2525,7 +2525,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G71" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="15" hidden="0" customHeight="1">
@@ -2546,7 +2546,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G72" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="15" hidden="0" customHeight="1">
@@ -2567,7 +2567,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G73" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="15" hidden="0" customHeight="1">
@@ -2588,7 +2588,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G74" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="15" hidden="0" customHeight="1">
@@ -2609,7 +2609,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G75" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="15" hidden="0" customHeight="1">
@@ -2630,7 +2630,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G76" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="15" hidden="0" customHeight="1">
@@ -2651,7 +2651,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G77" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="15" hidden="0" customHeight="1">
@@ -2672,7 +2672,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G78" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="15" hidden="0" customHeight="1">
@@ -2693,7 +2693,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G79" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="15" hidden="0" customHeight="1">
@@ -2714,7 +2714,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G80" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="15" hidden="0" customHeight="1">
@@ -2735,7 +2735,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G81" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="15" hidden="0" customHeight="1">
@@ -2756,7 +2756,7 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G82" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="15" hidden="0" customHeight="1">
@@ -2777,13 +2777,13 @@
         <x:v>MPN populated - verify source/availability</x:v>
       </x:c>
       <x:c r="G83" s="33" t="str">
-        <x:v>HOLD - DRC/parity not released</x:v>
+        <x:v>Review - owner signoff required</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfff543cfeb6b4721"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e1c7679c8ff4042"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2794,9 +2794,9 @@
   <x:cols>
     <x:col min="1" max="1" width="8.5" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="37" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="52.880001068115234" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="35.5" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="62" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="52" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
@@ -2841,13 +2841,13 @@
         <x:v>Design rules</x:v>
       </x:c>
       <x:c r="C3" s="33" t="str">
-        <x:v>943 native KiCad DRC violations</x:v>
+        <x:v>82 DRC warnings, 0 DRC errors, 0 unconnected items</x:v>
       </x:c>
       <x:c r="D3" s="33" t="str">
-        <x:v>Do not fabricate or assemble from current files</x:v>
+        <x:v>Rules review open on library/footprint mismatch warnings</x:v>
       </x:c>
       <x:c r="E3" s="33" t="str">
-        <x:v>Clean KiCad DRC</x:v>
+        <x:v>Resolve library mappings/footprints and rerun KiCad DRC</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -2858,13 +2858,13 @@
         <x:v>Shorts</x:v>
       </x:c>
       <x:c r="C4" s="33" t="str">
-        <x:v>43 shorting-item violations</x:v>
+        <x:v>Cleared in current cleanup</x:v>
       </x:c>
       <x:c r="D4" s="33" t="str">
-        <x:v>Electrical failure risk</x:v>
+        <x:v>No current shorting-item DRC errors reported</x:v>
       </x:c>
       <x:c r="E4" s="33" t="str">
-        <x:v>Re-layout/fix shorts and rerun DRC</x:v>
+        <x:v>Keep short checks in DRC regression before build authorization</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -2875,16 +2875,16 @@
         <x:v>Clearance</x:v>
       </x:c>
       <x:c r="C5" s="33" t="str">
-        <x:v>499 clearance violations</x:v>
+        <x:v>Cleared in current cleanup</x:v>
       </x:c>
       <x:c r="D5" s="33" t="str">
-        <x:v>Fabrication/electrical reliability risk</x:v>
+        <x:v>No current clearance DRC errors reported</x:v>
       </x:c>
       <x:c r="E5" s="33" t="str">
-        <x:v>Re-layout/fix clearances and rerun DRC</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
+        <x:v>Maintain constraints during schematic/netlist parity closure</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="24" hidden="0" customHeight="1">
       <x:c r="A6" s="33" t="str">
         <x:v>SCH-001</x:v>
       </x:c>
@@ -2892,16 +2892,16 @@
         <x:v>Schematic parity</x:v>
       </x:c>
       <x:c r="C6" s="33" t="str">
-        <x:v>564 parity issues</x:v>
+        <x:v>Open</x:v>
       </x:c>
       <x:c r="D6" s="33" t="str">
-        <x:v>Schematic/PCB mismatch risk</x:v>
+        <x:v>214 schematic-parity warnings remain because complete schematic/netlist source is missing</x:v>
       </x:c>
       <x:c r="E6" s="33" t="str">
-        <x:v>Resolve parity issues</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
+        <x:v>Import authoritative schematic/netlist and drive parity to zero</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="24" hidden="0" customHeight="1">
       <x:c r="A7" s="33" t="str">
         <x:v>MECH-001</x:v>
       </x:c>
@@ -2909,13 +2909,13 @@
         <x:v>Mechanical target</x:v>
       </x:c>
       <x:c r="C7" s="33" t="str">
-        <x:v>188.00 mm x 111.20 mm current board envelope</x:v>
+        <x:v>Current Edge.Cuts envelope approx. 305.0 mm x 260.5 mm; chassis constraints need confirmation</x:v>
       </x:c>
       <x:c r="D7" s="33" t="str">
-        <x:v>Confirm chosen server/MSI target before release</x:v>
+        <x:v>Confirm server/chassis target and mechanical envelope</x:v>
       </x:c>
       <x:c r="E7" s="33" t="str">
-        <x:v>Official mechanical signoff</x:v>
+        <x:v>Official chassis/mechanical signoff</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -2929,10 +2929,10 @@
         <x:v>Not passed</x:v>
       </x:c>
       <x:c r="D8" s="33" t="str">
-        <x:v>Fabricator review cannot be final</x:v>
+        <x:v>Fabricator review requires current Gerber/drill and stackup review</x:v>
       </x:c>
       <x:c r="E8" s="33" t="str">
-        <x:v>Clean DRC and fabricator DFM pass</x:v>
+        <x:v>DFM review using post-cleanup Gerber/drill package</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -2946,16 +2946,16 @@
         <x:v>Not passed</x:v>
       </x:c>
       <x:c r="D9" s="33" t="str">
-        <x:v>Assembly release blocked</x:v>
+        <x:v>Build authorization requires engineering signoff</x:v>
       </x:c>
       <x:c r="E9" s="33" t="str">
-        <x:v>Final BOM + placement + assembly validation</x:v>
+        <x:v>BOM + placement + assembly validation</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4228b7180114e4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b14cae274084a0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2976,7 +2976,7 @@
   <x:sheetData>
     <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
       <x:c r="A1" s="24" t="str">
-        <x:v>URGENT MANUFACTURER NOTICE - BOM AND BUILD HOLD</x:v>
+        <x:v>MANUFACTURER NOTICE - BOM AND GERBER REVIEW</x:v>
       </x:c>
       <x:c r="B1" s="25"/>
     </x:row>
@@ -2986,7 +2986,7 @@
     </x:row>
     <x:row r="3" ht="120" customHeight="1">
       <x:c r="A3" s="34" t="str">
-        <x:v>Use the Grouped BOM sheet as the current schematic-derived MPN list only. This is not a final verified procurement BOM release. The current July_04 design package is under fabrication and assembly hold because native KiCad DRC reports 943 violations, including 43 shorts and 499 clearance violations, and schematic parity reports 564 issues. If manufacturing has already started, pause procurement, fabrication, and assembly until engineering issues a clean DRC/parity result and final verified BOM signoff.</x:v>
+        <x:v>Use the Grouped BOM sheet as the current schematic-derived MPN list for the July_04 package. Current KiCad validation after non-netlist cleanup reports 0 DRC errors, 0 unconnected items, 82 library/footprint mismatch warnings, and 214 schematic-parity warnings. Engineering needs the complete schematic/netlist source to close parity; manufacturer review should focus on BOM/AVL, substitutions, stackup, drill/Gerber, and chassis-fit questions.</x:v>
       </x:c>
       <x:c r="B3" s="25"/>
     </x:row>
@@ -3059,7 +3059,7 @@
         <x:v>Release status</x:v>
       </x:c>
       <x:c r="B17" s="35" t="str">
-        <x:v>HOLD</x:v>
+        <x:v>ENGINEERING REVIEW</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
@@ -3138,7 +3138,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1f6c37d91754d82"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re885f893ac464b0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>